<commit_message>
登记 DD-70 / DD-71 与 IR-47 / IR-48
DD-70 发布形态：Ansible 剧本为权威来源，虚机镜像只能是剧本的派生产物；
离网介质自带 apt / PyPI / 容器三个仓库；构建期依赖不进墙内。
被拒绝方案里记下了「以镜像为交付物」的三条独立否决理由，其中第三条是
分发镜像会使我方成为 GPL 二进制的分发者（GPLv2 §3 / v3 §6），凭空产生
八年期的「提供对应源码」义务——交付剧本与校验和则什么都没分发。

DD-71 容器镜像跨墙用 skopeo + OCI 目录，复验锚点落在介质上的 manifest
而非本机镜像库；podman save/load 不保 digest（2026-10-08 实测，load 直接
拒绝）记入被拒绝方案。

IR-47 虚机按什么基线交付（决定 apt 闭包按什么底座解析，也决定能否发镜像）。
IR-48 介质导入流程，含「病毒扫描网关是否改写文件」——网关若重新打包压缩
文件，我方签名的 SHA256SUMS 与镜像 digest 复验会全部失败。建议正式交付前
做一次小样试导。

顺带修掉 HD-03 紧急度汇总表里一处陈旧计数（高 28 实际 31，现为 33），
并把正文的「共 45 项」更正为 48 项。

check_refs.py：悬空引用 0；CN 37 / DD 71 / AS 31 / IR 48 均无断号。

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MzPePSHWkTUSpnMTsqY5pZ
</commit_message>
<xml_diff>
--- a/HD-04_约束与设计决策登记册.xlsx
+++ b/HD-04_约束与设计决策登记册.xlsx
@@ -469,7 +469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A40"/>
+  <dimension ref="A1:A42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="150" customWidth="1" min="1" max="1"/>
@@ -677,6 +677,13 @@
       <c r="A40" t="inlineStr">
         <is>
           <t>【2026-10 补充】DD-69 记录 Python 依赖的两级冻结方式：Airflow 取上游官方 constraints（SHA-256 入 MANIFEST），dbt 由本方自维护 lock；两者统一离线安装。同轮修正了一处只在有网环境才看不出的缺陷——取料用的 pip download 虽不重复下载字节，却仍每次连 PyPI 重新解析依赖，剧本因此在真正离网的机器上跑不起来；现取料由 wheelhouse_refresh 开关控制，默认关闭。</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>【2026-10 补充】DD-70 与 DD-71 定下发布形态：权威来源是 Ansible 剧本而非虚机镜像，离网介质自带 apt / PyPI / 容器三个仓库，构建期依赖不进墙内（npm 这条供给链在生产网内因此不存在）。两条都来自 2026-10-08 在开发机上对交付路径的实测，而实测推翻了两处原本写进规程的做法：pip download 会把只发源码包的依赖原样带进墙内（改用 pip wheel），podman save/load 不保 digest 以致 load 直接拒绝（改用 skopeo + OCI 目录）。通用教训：交付路径上的每一个工具，都要在还有退路的时候实际跑一遍——开发机能上网这件事，会把离网问题推迟到最糟的时刻才暴露。IR-47（虚机基线）与 IR-48（介质导入流程与扫描网关是否改写文件）在答复前，介质的组织方式不能定稿。</t>
         </is>
       </c>
     </row>
@@ -1930,7 +1937,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H70"/>
+  <dimension ref="A1:H72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -4883,6 +4890,90 @@
         </is>
       </c>
     </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>DD-70</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>发布形态：Ansible 剧本为权威来源，虚机镜像只能是剧本的派生产物；离网介质自带 apt / PyPI / 容器三个仓库；构建期依赖不进墙内</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>MOI 生产网离网，且内网没有 apt 镜像、PyPI 镜像与容器镜像仓库。交付形态有两种候选：发一个装好的虚机镜像，还是发一套可执行的装配说明（剧本 + 物料）。八年合同期内还要持续打补丁。</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>一、权威来源是 infra/ 目录（剧本 + inventory + MANIFEST），镜像若出也必须由剧本跑出来，且纪律为「镜像里不许有剧本装不出来的东西」。二、介质自带三个仓库：签名的本地 apt 仓库（只含依赖闭包，非整源镜像）、wheelhouse（只含轮子）、OCI 目录（容器镜像）。三、区分构建期与运行期依赖，只有运行期依赖跨墙——门户前端的 Node/TypeScript 工具链不进生产网，只带编译产物 dist/，npm 这条供给链在墙内因此不存在。四、介质由剧本生成（90-bundle.yml），不手工攒。五、验收须在网卡真正禁用的全新虚机上、由另一个人重做一遍。做法记于 runbook/90-offline-media.md。</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>一、以虚机镜像为交付物（权威）。二、要求 MOI 在内网建三个仓库。三、把前端构建工具链一并带进生产网。</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>一、三条独立理由：①镜像把 OS 冻在打镜像那一刻，八年里每轮补丁要么让镜像作废要么要重走 MOI 审批（CN-13、CN-14）；②平台方若按自家基线交付虚机（IR-47），绕过其加固与补丁通道的自制镜像过不了安全审计；③分发镜像等于分发整个 Ubuntu 的 GPL 二进制，我方由此成为分发者并产生「提供对应源码」的持续义务（GPLv2 §3 / v3 §6）及修改版镜像的商标与再分发问题——而交付剧本与校验和则什么都没分发。二、不在我方可控范围，且把交付时点押在客户的基础设施建设上。三、带进墙内的每一样东西都是八年的维护义务；且构建失败的现场排查成本极高。</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>中（权威来源形态的改变会波及整个交付包的组织方式，但不涉及库结构与应用逻辑；镜像作为派生产物可随时增减）</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>REQ-OPS-01 · REQ-OPS-04 · CN-19 · DD-49 · DD-69 · IR-47 · IR-48</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>DD-71</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>容器镜像跨墙用 skopeo + OCI 目录传递，复验锚点落在介质上的 manifest 而非本机镜像库</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>镜像要随介质跨墙，而墙内没有镜像仓库。MANIFEST 以 digest 钉死镜像（DD-46 一线的纪律），但 digest 能否完整穿过介质此前从未实测。</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>一、用 skopeo copy --all 从仓库拷到介质上的 OCI 目录（manifest 逐字节拷贝，多架构 manifest list 一并带走）。二、现场复验用 skopeo inspect --raw &lt;OCI 目录&gt; | sha256sum，结果应等于 MANIFEST 记录的 digest——digest 的定义即 manifest 自身的 SHA-256，故该复验离网可做、不需要仓库、不信任任何中间环节。三、导入本机库时不得带 --all（containers-storage 存不下一组镜像），须以 --override-os/--override-arch 指定平台。四、skopeo 进 apt 闭包与 MANIFEST，墙内也要装。</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>一、podman save / podman load。二、不校验 digest，只校验归档文件的 SHA-256。</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>一、2026-10-08 在开发机实测：save --format oci-archive 之后 load 直接拒绝（Digest of source image's manifest would not match destination reference）。原因是上游 tag 为多架构 manifest list，而 save 只导出当前平台那一份，list 丢失后归档内容算出的 digest 与归档中记录的引用名不符。这不是配置问题，是该路径本身不保 digest。二、归档文件的哈希只能证明文件没在复制中损坏，证明不了它就是上游发布的那个镜像——与 ISO 校验必须先验签名再比哈希（MANIFEST「ISO 的校验方式」）是同一个道理。</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>低（传递工具与复验命令可更换，不影响镜像内容与运行形态；但复验锚点一旦改变须同步改写 MANIFEST 的纪律条文）</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>REQ-OPS-01 · CN-19 · DD-46 · DD-70 · T-15</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H28"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
DD-85 ETL 节点上的 Airflow 双活；LD-08 新增 3.3；资源表与 CLAUDE.md 同步
ETL-1、ETL-2 两台都运行 Airflow 全部组件（LocalExecutor），scheduler 不保存
状态，靠元数据库行锁协调，同一任务不会被两边同时执行；一台失效，其任务心跳
超时后由另一台重跑。

对任务的三条要求：能重跑；不依赖在哪台机器上运行（只经数据库或对象存储交接，
不经本地文件——单机开发环境里永远暴露不出来）；并发受限者用 pool。pool 是
元数据库中的一行，整个集群共用，不是每台各一：icp_cms、dbt_build 各 1 槽。
pool 只管经 Airflow 启动的任务，手工补数会绕过它，故接入程序另按源持有
PostgreSQL 咨询锁（经会话池，DD-67）。

被拒绝：CeleryExecutor（多一个须高可用的消息中间件）、主备加 VIP（自建切换、
双主风险）、只靠 pool（挡不住手工执行）。

资源表 ETL-1..2 的备注写明运行 Airflow（含组件与双活）、dbt 与接入作业；
CLAUDE.md 硬约束由五条增为七条。

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MzPePSHWkTUSpnMTsqY5pZ
</commit_message>
<xml_diff>
--- a/HD-04_约束与设计决策登记册.xlsx
+++ b/HD-04_约束与设计决策登记册.xlsx
@@ -469,7 +469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A54"/>
+  <dimension ref="A1:A56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="150" customWidth="1" min="1" max="1"/>
@@ -547,6 +547,7 @@
         </is>
       </c>
     </row>
+    <row r="13"/>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
@@ -624,6 +625,7 @@
         </is>
       </c>
     </row>
+    <row r="25"/>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
@@ -631,6 +633,7 @@
         </is>
       </c>
     </row>
+    <row r="27"/>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
@@ -638,6 +641,7 @@
         </is>
       </c>
     </row>
+    <row r="29"/>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
@@ -645,6 +649,7 @@
         </is>
       </c>
     </row>
+    <row r="31"/>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
@@ -652,6 +657,7 @@
         </is>
       </c>
     </row>
+    <row r="33"/>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
@@ -659,6 +665,7 @@
         </is>
       </c>
     </row>
+    <row r="35"/>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
@@ -666,6 +673,7 @@
         </is>
       </c>
     </row>
+    <row r="37"/>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
@@ -673,6 +681,7 @@
         </is>
       </c>
     </row>
+    <row r="39"/>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
@@ -680,6 +689,7 @@
         </is>
       </c>
     </row>
+    <row r="41"/>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
@@ -687,6 +697,7 @@
         </is>
       </c>
     </row>
+    <row r="43"/>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
@@ -694,6 +705,7 @@
         </is>
       </c>
     </row>
+    <row r="45"/>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
@@ -701,6 +713,7 @@
         </is>
       </c>
     </row>
+    <row r="47"/>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
@@ -708,6 +721,7 @@
         </is>
       </c>
     </row>
+    <row r="49"/>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
@@ -715,6 +729,7 @@
         </is>
       </c>
     </row>
+    <row r="51"/>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
@@ -722,10 +737,18 @@
         </is>
       </c>
     </row>
+    <row r="53"/>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
           <t>【2026-10 补充】DD-82 解决 ICP 契约与 raw 只追加的冲突，并防止 raw 因回看而膨胀 4 至 5 倍：只追加有变化的观测，去重不计被扣下的批次。DD-83 与开发机发现的镜像 digest 问题同源——lock 两份、constraints 校验和只打印不比对，都是「只在纸面上钉死」。钉死一个值，必须有一个环节在它不符时失败，否则写下的值只是注释。</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>【2026-10 补充】DD-84 与 DD-85 定下接入程序的形态与 ETL 节点的高可用。DD-85 补上 LD-08 的一处空白：此前只写了 ETL「成对部署」，没有写两台如何配合。双活成立的前提是 scheduler 无状态，而对任务的要求是能重跑、不依赖在哪台机器上运行、并发受限者用全局 pool——其中第二条在单机开发环境里永远不会暴露。</t>
         </is>
       </c>
     </row>
@@ -1979,7 +2002,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H85"/>
+  <dimension ref="A1:H86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -5562,6 +5585,48 @@
         </is>
       </c>
     </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>DD-85</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>ETL-1、ETL-2 上的 Airflow 双活：两台均运行全部组件，LocalExecutor，靠元数据库行锁协调；任务须能重跑、不依赖在哪台机器上运行、并发受限者用全局 pool 约束</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>资源表中 ETL-1..2 只写「Batch orchestration and model builds」，未写明运行 Airflow 与 dbt；LD-08 只写「成对部署」与「跨两台物理主机」（PL-03），没有设计两台如何配合、一台失效会怎样（2026-10-13 Gavin 指出）。</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>一、两台都运行 api-server、scheduler、dag-processor、triggerer，执行器 LocalExecutor，元数据库在 PostgreSQL 集群中的独立数据库（DD-44）。二、scheduler 不保存状态，任务依赖、实例状态与 pool 占用都在元数据库，两个 scheduler 以行锁协调，同一任务不会被两边同时执行。三、一台失效时，其上运行中的任务心跳超时后被标为失败，按重试由另一台重跑。四、任务须满足：能重跑；不依赖在哪台机器上运行——任务之间只经数据库或对象存储交接，不经本地文件；并发受限者用 pool 约束。五、pool icp_cms 与 dbt_build 各 1 个槽位；pool 为全局，非每台各一。六、接入程序另按源持有 PostgreSQL 咨询锁（经会话池），使手工补数也不会与定时任务并发取数。七、测试环境安排一次双节点验证。详见 LD-08 3.3。</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>一、CeleryExecutor。二、主备加虚拟 IP 切换。三、只靠 pool 防止 ICP 并发下载。</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>一、须多一个消息中间件（Redis 或 RabbitMQ），其自身又要做高可用，是又一个须维护八年的组件；本项目的任务量用不着分布式执行。二、要自建故障切换并承担双主风险；Airflow 本身支持多个 scheduler 同时工作，无需另设选主机制。三、pool 只约束经 Airflow 启动的任务，按 DD-84 接入程序可手工执行补数，手工那一次绕过 pool。</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>中（执行器与部署形态改动涉及两台的配置与剧本；三条任务要求一旦被违反，错误为间歇性，难以复现）</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>REQ-AVL-01 · REQ-OPS-01 · PL-03 · DD-44 · DD-67 · DD-82 · DD-84</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H28"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
DD-91 core 装载规则十二处、DD-92 caller_number_hash；LD-02 第 3 章补充段；LD-10 用例改号 TC-DISC-19/20/21；AS-32/33 更正；NOTES 回复 dbt 方案
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MzPePSHWkTUSpnMTsqY5pZ
</commit_message>
<xml_diff>
--- a/HD-04_约束与设计决策登记册.xlsx
+++ b/HD-04_约束与设计决策登记册.xlsx
@@ -469,7 +469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A68"/>
+  <dimension ref="A1:A69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="150" customWidth="1" min="1" max="1"/>
@@ -817,6 +817,13 @@
       <c r="A68" t="inlineStr">
         <is>
           <t>2026-10-26：DD-73/74/85/89/90 加注（cad_mirror 独立序列与开发期重建、CONNECT 收回、密钥权威来源、resweep 逻辑日期、触发器与改名列）；规范 v0.6。</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2026-10-27：新增 DD-91（core 装载规则十二处）、DD-92（caller_number_hash 算法，先留空）；LD-10 三条用例编号改为 TC-DISC-19/20/21（原编号与 test/cases_seed.csv 冲突）。</t>
         </is>
       </c>
     </row>
@@ -2070,7 +2077,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H91"/>
+  <dimension ref="A1:H93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -5419,7 +5426,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>一、发生日语义（发生类指标、按发生时间检索）：同时带 date_key 范围与时间列范围。二、关闭日语义（结案类指标、按关闭时间检索）：不加 date_key 下界，只可加安全上界 date_key &lt;= 结束日，由 closed_date_key 索引定位。三、结案类指标的查询 API 走按关闭日聚合的 mart。四、指标属哪一类以 LD-03 分类与指标注册表为准，服务层不自行判断。五、LD-10 增加纪律用例 TC-DISC-04（跨月与跨年关闭）。</t>
+          <t>一、发生日语义（发生类指标、按发生时间检索）：同时带 date_key 范围与时间列范围。二、关闭日语义（结案类指标、按关闭时间检索）：不加 date_key 下界，只可加安全上界 date_key &lt;= 结束日，由 closed_date_key 索引定位。三、结案类指标的查询 API 走按关闭日聚合的 mart。四、指标属哪一类以 LD-03 分类与指标注册表为准，服务层不自行判断。五、LD-10 增加纪律用例 TC-DISC-19（跨月与跨年关闭）。</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
@@ -5797,7 +5804,7 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>一、同步由部署做：40-schema 之后新增一步，以属主身份把 contracts/ 下的 YAML 写入 meta.source_contract，只写 definition、contract_version、target_raw、connector，且只在文件版本号大于库内时写（向前不向后，与 LD-08 7.2 同一规则）。二、新建 meta.source_runtime_param（source_id、参数名、值、更新时间、更新人），M-01 的四类热调项（启停、间隔、批量、限流）写这里并留痕于 audit.runtime_param_change_log；enabled 列属启停，同步永不触碰。接入程序读 definition 再叠加 runtime_param。三、新结构变更把 admin_svc 对 source_contract 的 UPDATE 收窄为 UPDATE (enabled)，其余撤销（0002 已执行，不改原文件）。四、raw 表按月分区，键为 ingested_at，索引按 DD-78（见 LD-02 第 9 章）。 ——【2026-10-18 同日评审更正，按 DD-51 先例原地改】五、meta.quarantine_batch 的外键由 run_log 改指向 meta.ingest_batch (run_id, batch_seq)：批次先提交、run_log 最后写，第一批若需隔离时父记录尚不存在。六、有效配置在运行开始时解析一次、整个运行沿用，热调项快照写入 ingest_batch.effective_params；热调白名单（参数名、类型、范围）写入 source_runtime_param 的 CHECK；启停只认 source_contract.enabled，白名单不含启停；第一版轮询间隔为发布项、不可热调（接入程序读参数改变不了 DAG 触发频率，LD-06 2.4 随之更正）。七、契约同步分三支：同版本同内容不动、同版本不同内容部署失败并提示递增版本、文件版本低于库内拒绝；新版本同步前按新白名单校验既有热调值，不兼容则部署失败列出参数，不自动作废。八、内容哈希覆盖实际收到的完整字段名与原值，不限于契约已登记列。九、分区去重性能列为待验证（LD-10 TC-ING-01），不预先宣布可接受。 ——【2026-10-19 0004 落地补记】十、meta.ensure_monthly_partitions 的范围由 core · audit 扩大到 raw（0002 曾收窄；raw 按月分区后须以属主身份建分区，接入角色不得自建）；timestamptz 分区键 ingested_at 的月边界取 UTC 月初零点并带显式偏移——它是系统时间，无业务日含义，不适用 LD-02 第 6 章的归日时区。十一、meta.run_log.outcome 只表达提交状态：success / partial / failed；quarantined 不再使用但不改 CHECK，隔离情况由 M-01 关联 meta.quarantine_batch 呈现，不混入 outcome。十二、热调白名单第一版只有 lookback_minutes（1–1440）；批量与限流待第一份用到它们的契约随结构变更加入。十三、ingest_batch 另有 rows_written 与 received_header 两列；raw 每行带指向 ingest_batch 的外键。 ——【2026-10-19 评审第四轮】十四、契约校验只有一套，在接入程序内，部署与 M-01 调用它；最小校验集与 YAML 重复键拒绝见 LD-01 2.5。十五、热调的回看长度只能调大、不得小于契约默认值（缩短只少数据不报错）；调小走发布。0004 的 CHECK 不改，规则在校验代码里。十六、契约同步事务加 pg_advisory_xact_lock 串行化。 ——【2026-10-21 评审第五轮】十七、部署同步对契约行 FOR UPDATE、M-01 对同一行 FOR SHARE，堵住部署与热调之间的竞态（advisory lock 只管部署之间）；十八、接入启动时契约与覆盖值同一快照读取；十九、校验分通用层与按连接器的必填层，必填缺失为配置错误、退出码 2。</t>
+          <t>一、同步由部署做：40-schema 之后新增一步，以属主身份把 contracts/ 下的 YAML 写入 meta.source_contract，只写 definition、contract_version、target_raw、connector，且只在文件版本号大于库内时写（向前不向后，与 LD-08 7.2 同一规则）。二、新建 meta.source_runtime_param（source_id、参数名、值、更新时间、更新人），M-01 的四类热调项（启停、间隔、批量、限流）写这里并留痕于 audit.runtime_param_change_log；enabled 列属启停，同步永不触碰。接入程序读 definition 再叠加 runtime_param。三、新结构变更把 admin_svc 对 source_contract 的 UPDATE 收窄为 UPDATE (enabled)，其余撤销（0002 已执行，不改原文件）。四、raw 表按月分区，键为 ingested_at，索引按 DD-78（见 LD-02 第 9 章）。 ——【2026-10-18 同日评审更正，按 DD-51 先例原地改】五、meta.quarantine_batch 的外键由 run_log 改指向 meta.ingest_batch (run_id, batch_seq)：批次先提交、run_log 最后写，第一批若需隔离时父记录尚不存在。六、有效配置在运行开始时解析一次、整个运行沿用，热调项快照写入 ingest_batch.effective_params；热调白名单（参数名、类型、范围）写入 source_runtime_param 的 CHECK；启停只认 source_contract.enabled，白名单不含启停；第一版轮询间隔为发布项、不可热调（接入程序读参数改变不了 DAG 触发频率，LD-06 2.4 随之更正）。七、契约同步分三支：同版本同内容不动、同版本不同内容部署失败并提示递增版本、文件版本低于库内拒绝；新版本同步前按新白名单校验既有热调值，不兼容则部署失败列出参数，不自动作废。八、内容哈希覆盖实际收到的完整字段名与原值，不限于契约已登记列。九、分区去重性能列为待验证（LD-10 TC-DISC-20），不预先宣布可接受。 ——【2026-10-19 0004 落地补记】十、meta.ensure_monthly_partitions 的范围由 core · audit 扩大到 raw（0002 曾收窄；raw 按月分区后须以属主身份建分区，接入角色不得自建）；timestamptz 分区键 ingested_at 的月边界取 UTC 月初零点并带显式偏移——它是系统时间，无业务日含义，不适用 LD-02 第 6 章的归日时区。十一、meta.run_log.outcome 只表达提交状态：success / partial / failed；quarantined 不再使用但不改 CHECK，隔离情况由 M-01 关联 meta.quarantine_batch 呈现，不混入 outcome。十二、热调白名单第一版只有 lookback_minutes（1–1440）；批量与限流待第一份用到它们的契约随结构变更加入。十三、ingest_batch 另有 rows_written 与 received_header 两列；raw 每行带指向 ingest_batch 的外键。 ——【2026-10-19 评审第四轮】十四、契约校验只有一套，在接入程序内，部署与 M-01 调用它；最小校验集与 YAML 重复键拒绝见 LD-01 2.5。十五、热调的回看长度只能调大、不得小于契约默认值（缩短只少数据不报错）；调小走发布。0004 的 CHECK 不改，规则在校验代码里。十六、契约同步事务加 pg_advisory_xact_lock 串行化。 ——【2026-10-21 评审第五轮】十七、部署同步对契约行 FOR UPDATE、M-01 对同一行 FOR SHARE，堵住部署与热调之间的竞态（advisory lock 只管部署之间）；十八、接入启动时契约与覆盖值同一快照读取；十九、校验分通用层与按连接器的必填层，必填缺失为配置错误、退出码 2。</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
@@ -5881,7 +5888,7 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>一、接受，但结构必须是 CAD 原样（Table Lists 英文视图名、翻译列名、全部列不筛选），DDL 由 DS 定义与交付、本方只审不改——这与 DD-04 否掉的方案差一个词：那是我方模型由 DS 映射，这是源端原样换个地方放，raw「源端交来什么就记什么」不变。二、同集群单独 database cad_mirror（Gavin 2026-10-19 定），写入角色 cad_mirror_writer 仅为该库属主，对 oss911 零权限；经 pgBouncer session 模式单独池写入。三、写入方式按主键 UPSERT，不 TRUNCATE、不整表重载；DS 每周期写心跳表。四、每表加 mirror_updated_at 列由触发器维护，作为水位列，sjc 不可靠（Q10）由此解决；8.3 滚动窗口校验降回加固措施。五、中间库即交接点，中间库与 CAD 一致由 DS 负责；DS 定期提供 CAD 源端按日计数供本方对账。六、入向网络通道须 MOI 批（IR-52）。七、规范发 DS 会签（queries/CAD_Mirror_Database_Specification.docx），空白项为 IR-51。 ——【2026-10-19 同日评审更正，原地改】四、触发器时间戳不是提交时间（now() 更是事务开始时间），不能据此把回扫降级：窗口上界改取最新心跳的 started_at（DS 周期串行、心跳后写，故为提交围栏）；writer 角色设 statement_timeout 与 idle_in_transaction_session_timeout；8.3 回扫维持必需项，待 TC-ING-02 通过再议。二、写入角色不是属主：cad_mirror 由 NOLOGIN 的 cad_mirror_owner 持有，cad_mirror_writer 只有 CONNECT、USAGE、cad.* 的 SELECT/INSERT/UPDATE、cad_meta.* 的 INSERT，无 CREATE/DELETE/TRUNCATE/TRIGGER。 ——【2026-10-19 补记】CAD 自身的库为 PostgreSQL（SQL Server 为上一代 BI 附带的中间层），中间库 DDL 不需要跨产品转换：取 CAD 原库 PG DDL 原样、只改名。规范 v0.3 的 3.6 节（SQL Server→PG 十处差异）在 v0.4 中撤回，IR-51 相应更正。 ——【2026-10-25 更正条件一】上一代中间库的 DDL 由当时的 BI 方建、DS 只写入（Gavin 告知），故 DDL 改为由本方按《Bill同步CAD表数据结构》生成、DS 核对会签。DD-04 的边界由此只能靠本方自律：74 张表全部列照建、一列不少、不加任何本方模型的东西；类型映射宁宽勿严（text / timestamp / numeric），收紧放在 staging。另向 DS 索取 CAD 原库完整目录，判断结构表是否为上一代 BI 选定的子集。 ——【2026-10-26 注】触发器对内容相同的 UPDATE 不写新行版本、不动时间戳（DD-78 的同一原则），UPSERT 因此回报 0 行是有意的，已写进规范 v0.6；21 个保留字列名改名不加引号，两处重名列待 DS 给译名；水位列改 B-tree（UPSERT 原地改写）。</t>
+          <t>一、接受，但结构必须是 CAD 原样（Table Lists 英文视图名、翻译列名、全部列不筛选），DDL 由 DS 定义与交付、本方只审不改——这与 DD-04 否掉的方案差一个词：那是我方模型由 DS 映射，这是源端原样换个地方放，raw「源端交来什么就记什么」不变。二、同集群单独 database cad_mirror（Gavin 2026-10-19 定），写入角色 cad_mirror_writer 仅为该库属主，对 oss911 零权限；经 pgBouncer session 模式单独池写入。三、写入方式按主键 UPSERT，不 TRUNCATE、不整表重载；DS 每周期写心跳表。四、每表加 mirror_updated_at 列由触发器维护，作为水位列，sjc 不可靠（Q10）由此解决；8.3 滚动窗口校验降回加固措施。五、中间库即交接点，中间库与 CAD 一致由 DS 负责；DS 定期提供 CAD 源端按日计数供本方对账。六、入向网络通道须 MOI 批（IR-52）。七、规范发 DS 会签（queries/CAD_Mirror_Database_Specification.docx），空白项为 IR-51。 ——【2026-10-19 同日评审更正，原地改】四、触发器时间戳不是提交时间（now() 更是事务开始时间），不能据此把回扫降级：窗口上界改取最新心跳的 started_at（DS 周期串行、心跳后写，故为提交围栏）；writer 角色设 statement_timeout 与 idle_in_transaction_session_timeout；8.3 回扫维持必需项，待 TC-DISC-21 通过再议。二、写入角色不是属主：cad_mirror 由 NOLOGIN 的 cad_mirror_owner 持有，cad_mirror_writer 只有 CONNECT、USAGE、cad.* 的 SELECT/INSERT/UPDATE、cad_meta.* 的 INSERT，无 CREATE/DELETE/TRUNCATE/TRIGGER。 ——【2026-10-19 补记】CAD 自身的库为 PostgreSQL（SQL Server 为上一代 BI 附带的中间层），中间库 DDL 不需要跨产品转换：取 CAD 原库 PG DDL 原样、只改名。规范 v0.3 的 3.6 节（SQL Server→PG 十处差异）在 v0.4 中撤回，IR-51 相应更正。 ——【2026-10-25 更正条件一】上一代中间库的 DDL 由当时的 BI 方建、DS 只写入（Gavin 告知），故 DDL 改为由本方按《Bill同步CAD表数据结构》生成、DS 核对会签。DD-04 的边界由此只能靠本方自律：74 张表全部列照建、一列不少、不加任何本方模型的东西；类型映射宁宽勿严（text / timestamp / numeric），收紧放在 staging。另向 DS 索取 CAD 原库完整目录，判断结构表是否为上一代 BI 选定的子集。 ——【2026-10-26 注】触发器对内容相同的 UPDATE 不写新行版本、不动时间戳（DD-78 的同一原则），UPSERT 因此回报 0 行是有意的，已写进规范 v0.6；21 个保留字列名改名不加引号，两处重名列待 DS 给译名；水位列改 B-tree（UPSERT 原地改写）。</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
@@ -5902,6 +5909,90 @@
       <c r="H91" t="inlineStr">
         <is>
           <t>REQ-ING-02 · DD-02 · DD-04 · DD-58 · DD-61 · DD-74 · IR-02 · IR-50 · IR-51 · IR-52 · LD-01 第 3 章 · LD-07 2.1 · LD-08 第 8 章</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>DD-91</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>core 装载规则十二处：src_system 按系统取值（icp · cad · cad_archive）、站点 MKK 以结构变更写入、维度迟到留空不造成员、CHECK 增 unmapped、释放原因归类进契约、src_observed_at 与派生内容哈希决定写入、date_key 变化按 sk 跨分区先删后插、transform 可写待澄清队列、tz 偏移取契约约定、分区预建三个月、dbt 独立 DAG 同频运行</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>开发机写 dbt 前逐条核对 LD-02、DD-06/66/74/77/78/79/82/89 与契约，发现十二处设计空白或冲突，其中代理键的 src_system 一经上线不可改（2026-10-26 NOTES）。</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>见 LD-02 第 3 章末补充段的十二条。要点：src_system 按系统不按源，使同一系统的坐席工号在维度与事实上算出同一键；归档单独为 cad_archive，以免割接并行期与 CAD 撞键；unmapped 是 DD-06「未映射不得归入其他」在 CHECK 上的落实；写入判定按 core 行派生内容而非源端原文，否则归类表更正与维度补齐永远写不进去；dbt 不接在增量 DAG 之后，因同一 DAG 内 max_active_runs = 1 会让 dbt 重试堵住接入。</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>一、src_system 按源（icp_cdr_voice）。二、维度缺席时造「未知坐席」占位成员。三、CHECK 不加 unmapped，值表外归 internal。四、dbt 作为增量 DAG 的第二个任务。</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>一、同一坐席在话单与参照数据里会算出两个键。二、占位成员会被当成真实维度成员统计，且 dim 的 NOT NULL 列只能编造。三、违反 DD-06，已知内部呼叫与未知码混在一起。四、耦合失败路径：dbt 失败重试期间接入停摆。</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>低至中（多为 dbt 模型与两个小结构变更；src_system 与 site_code 一旦有数据即不可逆）</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>DD-06 · DD-60 · DD-74 · DD-77 · DD-78 · DD-82 · DD-89 · LD-02 第 3、4、6、9 章 · LD-01 4.3 · if03a</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>DD-92</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>caller_number_hash 的算法定为 HMAC-SHA256（密钥只存 /etc/oss911，不入库），规范化后计算；本批先留空，密钥传入 dbt 的路径随 LD-07 那批设计</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>fact_call_leg.caller_number_hash 无算法、盐与规范化规则（DD-35 敏感字段）。不加盐的号码哈希可穷举还原；CALLERNO 可为邮件或网址。M-C15 以它为分组键。</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>一、算法 HMAC-SHA256，密钥由剧本生成、存 /etc/oss911（0600）、不入库、不入契约。二、规范化：数字串去掉非数字并去前导 00 / +，其余（邮件、网址）小写去首尾空白，前缀类型标记（n: / e: / u:）后再计算。三、core 保留 caller_number 明文列（受 DD-35 可见性矩阵约束），故哈希可随时按新密钥或新规则整体重算，历史不会断档——这是本步可以先留空的依据。四、dbt 取密钥的路径（不经 dbt 变量进入日志）在 LD-07 的实现批次定，定下即补算。</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>一、SHA-256 不加盐。二、现在随手定一个算法先写入。三、不存哈希，M-C15 直接按明文分组。</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>一、11 位号码空间可在普通硬件上穷举还原，等于没有保护。二、密钥传入路径没想清楚就实现，密钥会出现在 dbt 日志或 manifest 里。三、分组查询必须能读明文列，等于把 M-C15 的使用者全部提升到可见号码的角色。</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>低（留空列，后补；重算可行）</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>DD-35 · REQ-GOV-02 · M-C15 · LD-07 2.2 · LD-02 第 3 章</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
DD-94 补记 requested_from / cleared_by 与按字段留痕
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MzPePSHWkTUSpnMTsqY5pZ
</commit_message>
<xml_diff>
--- a/HD-04_约束与设计决策登记册.xlsx
+++ b/HD-04_约束与设计决策登记册.xlsx
@@ -469,7 +469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A74"/>
+  <dimension ref="A1:A75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="150" customWidth="1" min="1" max="1"/>
@@ -859,6 +859,13 @@
       <c r="A74" t="inlineStr">
         <is>
           <t>2026-10-29：DD-94 补记开发机十一处（一处更正：角色标记版本的留痕 changed_by 取操作人）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>2026-10-29：DD-94 补记 requested_from / cleared_by 与按字段留痕。</t>
         </is>
       </c>
     </row>
@@ -6091,7 +6098,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>一、经 raw（raw.icp_reference，通用列 + payload 原样）；LD-01 9.3 收窄为「M-10 人工维护的不经 raw」。二、版本变了整份快照写入，每数据集一批，core 以最新快照判消失；契约 raw_write.mode 改 snapshot_on_version。三、vdns 用 CTI 版本、其余用 VDN 版本，水位按 (ccId, vdnId)；只在 status = 2 取数。四、不调 syncti / synvdn；endTime 超 N 天（首版 7，热调 version_stale_days）未变告警；Q33 问网关是否自动同步。五、valid_from 取同步 endTime，首版取哨兵（早于一切事实；sk_scd 须能表示）。六、【2026-10-27 同日更正，Gavin 告知 ICP 的工号只有接警员与其主管、调度员不接电话（AS-36）】ICP 同步的坐席 role_code 默认 call_taker；主管由 M-10 标记为 supervisor（SCD2 留痕）；调度员的维度行将来自 CAD 上下岗记录，不经 ICP。Q35 仍问 ICP，不再阻塞。七、team_code 取 groupId，组名进 reference_value，monitorId 不落 core。八、dim_queue 双语列先写 skillName 原文，译名走 label_override。九、技能组多对多：skill_group_code 留空，成员关系只在 raw，需要时立桥表。十、calledconfigs 只落 raw，不进 dim_channel；落点待有指标需要时定。十一、oss911_transform 获 dim_agent / dim_queue 的 INSERT 与 UPDATE(valid_to, built_at)、reference_value 的 INSERT / UPDATE、reference_data_change_log 的 INSERT、label_override 的 UPDATE(state, flagged_at)。十二、版本更小由接入程序判、进待澄清；版本变而内容无差异由 dbt 判、记日志告警。十三、全部技能入 dim_queue，realFlag 只在 raw。十四、agentName 空或等于工号照写原文。 ——【2026-10-28 评审更正，原地改】十五、快照型数据集只要有一条缺自然键的记录即整批隔离（raw 照存），不得用不完整的快照做「消失即置非当前」的判断；全部缺键同样隔离。十六、M-10 的主管标记存为带生效区间的变更记录 meta.agent_role_override（agent_no、role_code、valid_from、valid_to、changed_by、reason），撤销是关 valid_to 不删行；dbt 按源端快照与 M-10 两类变化点的并集切 SCD2 版本，不同生效时刻的变化不合成一版（LD-02 第 7 章新增规则）。十七、staging 只处理契约配置的 VDN；其他 VDN 的快照留 raw 并进待澄清，不进维度模型；AS-30 被推翻时按其影响条款加 VDN 维，不现在把 vdn_id 塞进自然键。 ——【2026-10-28 开发机实现中定的十四处，知悉并登记】已取版本记在 ingest_batch 的 snapshot_scope / snapshot_version / snapshot_synced_at，不写 watermark_state；隔离中的批次也算已取；首版哨兵 1970-01-01 UTC（-infinity 经 to_char 得 NULL）；副本过期只写 run_log message「STALE:」，监控批次接告警；reference_value 增 src_label、last_seen_at 改为最近变化时刻；每次构建只应用一份快照、从旧到新；已有话单由维度模型 post-hook 只对涉及的成员重新关联；dim_agent 名称两列同样先写原文；dbt 覆盖 get_columns_in_relation 跳过生成列；「版本变而内容无差异」为 warn 级 dbt 测试；transform 获 audit 的 USAGE；version_stale_days 可升可降。其中「缺键照写不隔离」「撤销即删行」「多 VDN 照常进维度」三处已被十五至十七推翻。 ——【2026-10-29 开发机实现中定的十一处，知悉并登记】一次构建应用全部待应用快照（变化点并集所需）；补登过去的角色标记从该成员最新版本之后一秒生效、不改写已生效版本，M-10 录入时显示「将从 X 起生效」并要求确认、记录保留 requested_from；起点在将来的标记到点后才切版；agent_role_override 带 site_code / src_system / override_id / recorded_at，同一成员区间不重叠用排他约束（btree_gist 由 20-database 建，真机先 20 后 40）；M-10 只能 INSERT 与 UPDATE(valid_to)；标记引起的维度版本留痕 changed_by 取标记的操作人、reason「(role mark)」，icp_sync 只用于源端驱动的版本（更正开发机原定）；契约 v3 增 endpoint.site_vdn 必填，开发值随发布进生产，列入发布核对清单必核项；出现 site_vdn 以外的 VDN 或 site_vdn 不在版本号里各开待澄清；staging 不登记其他 VDN 的批次；DD-95 待澄清由 fact_call_leg 与两个维度模型的 post-hook 开、归 icp_reference；mart 的 unlinked 桶随 fact_call 一批实现。</t>
+          <t>一、经 raw（raw.icp_reference，通用列 + payload 原样）；LD-01 9.3 收窄为「M-10 人工维护的不经 raw」。二、版本变了整份快照写入，每数据集一批，core 以最新快照判消失；契约 raw_write.mode 改 snapshot_on_version。三、vdns 用 CTI 版本、其余用 VDN 版本，水位按 (ccId, vdnId)；只在 status = 2 取数。四、不调 syncti / synvdn；endTime 超 N 天（首版 7，热调 version_stale_days）未变告警；Q33 问网关是否自动同步。五、valid_from 取同步 endTime，首版取哨兵（早于一切事实；sk_scd 须能表示）。六、【2026-10-27 同日更正，Gavin 告知 ICP 的工号只有接警员与其主管、调度员不接电话（AS-36）】ICP 同步的坐席 role_code 默认 call_taker；主管由 M-10 标记为 supervisor（SCD2 留痕）；调度员的维度行将来自 CAD 上下岗记录，不经 ICP。Q35 仍问 ICP，不再阻塞。七、team_code 取 groupId，组名进 reference_value，monitorId 不落 core。八、dim_queue 双语列先写 skillName 原文，译名走 label_override。九、技能组多对多：skill_group_code 留空，成员关系只在 raw，需要时立桥表。十、calledconfigs 只落 raw，不进 dim_channel；落点待有指标需要时定。十一、oss911_transform 获 dim_agent / dim_queue 的 INSERT 与 UPDATE(valid_to, built_at)、reference_value 的 INSERT / UPDATE、reference_data_change_log 的 INSERT、label_override 的 UPDATE(state, flagged_at)。十二、版本更小由接入程序判、进待澄清；版本变而内容无差异由 dbt 判、记日志告警。十三、全部技能入 dim_queue，realFlag 只在 raw。十四、agentName 空或等于工号照写原文。 ——【2026-10-28 评审更正，原地改】十五、快照型数据集只要有一条缺自然键的记录即整批隔离（raw 照存），不得用不完整的快照做「消失即置非当前」的判断；全部缺键同样隔离。十六、M-10 的主管标记存为带生效区间的变更记录 meta.agent_role_override（agent_no、role_code、valid_from、valid_to、changed_by、reason），撤销是关 valid_to 不删行；dbt 按源端快照与 M-10 两类变化点的并集切 SCD2 版本，不同生效时刻的变化不合成一版（LD-02 第 7 章新增规则）。十七、staging 只处理契约配置的 VDN；其他 VDN 的快照留 raw 并进待澄清，不进维度模型；AS-30 被推翻时按其影响条款加 VDN 维，不现在把 vdn_id 塞进自然键。 ——【2026-10-28 开发机实现中定的十四处，知悉并登记】已取版本记在 ingest_batch 的 snapshot_scope / snapshot_version / snapshot_synced_at，不写 watermark_state；隔离中的批次也算已取；首版哨兵 1970-01-01 UTC（-infinity 经 to_char 得 NULL）；副本过期只写 run_log message「STALE:」，监控批次接告警；reference_value 增 src_label、last_seen_at 改为最近变化时刻；每次构建只应用一份快照、从旧到新；已有话单由维度模型 post-hook 只对涉及的成员重新关联；dim_agent 名称两列同样先写原文；dbt 覆盖 get_columns_in_relation 跳过生成列；「版本变而内容无差异」为 warn 级 dbt 测试；transform 获 audit 的 USAGE；version_stale_days 可升可降。其中「缺键照写不隔离」「撤销即删行」「多 VDN 照常进维度」三处已被十五至十七推翻。 ——【2026-10-29 开发机实现中定的十一处，知悉并登记】一次构建应用全部待应用快照（变化点并集所需）；补登过去的角色标记从该成员最新版本之后一秒生效、不改写已生效版本，M-10 录入时显示「将从 X 起生效」并要求确认、记录保留 requested_from；起点在将来的标记到点后才切版；agent_role_override 带 site_code / src_system / override_id / recorded_at，同一成员区间不重叠用排他约束（btree_gist 由 20-database 建，真机先 20 后 40）；M-10 只能 INSERT 与 UPDATE(valid_to)；标记引起的维度版本留痕 changed_by 取标记的操作人、reason「(role mark)」，icp_sync 只用于源端驱动的版本（更正开发机原定）；契约 v3 增 endpoint.site_vdn 必填，开发值随发布进生产，列入发布核对清单必核项；出现 site_vdn 以外的 VDN 或 site_vdn 不在版本号里各开待澄清；staging 不登记其他 VDN 的批次；DD-95 待澄清由 fact_call_leg 与两个维度模型的 post-hook 开、归 icp_reference；mart 的 unlinked 桶随 fact_call 一批实现。 ——【2026-10-29 补记】agent_role_override 增 requested_from（M-10 确认后 valid_from 写实际生效点、原申请起点留存）与 cleared_by（撤销人，仅 valid_to 非无穷时可填，M-10 获 UPDATE(cleared_by)）；撤销引起的版本留痕取 coalesce(cleared_by, changed_by)；留痕按字段分：role_code 行记标记操作人，源端字段与 is_current 记 icp_sync。被拒：另建撤销记录表；撤销改为插入 call_taker 标记（与十六条冲突，且「回到默认」与「明确标为接警员」无法区分）。</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">

</xml_diff>

<commit_message>
DD-96 fact_call 聚合规则与 call_result 四值（unanswered_system）；DD-97 注册表与 mart 对应、版本后缀；LD-03 2.4 与第 5 章补充；LD-02 第 10 章注；NOTES 第 8 步开工清单
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MzPePSHWkTUSpnMTsqY5pZ
</commit_message>
<xml_diff>
--- a/HD-04_约束与设计决策登记册.xlsx
+++ b/HD-04_约束与设计决策登记册.xlsx
@@ -469,7 +469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A76"/>
+  <dimension ref="A1:A77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="150" customWidth="1" min="1" max="1"/>
@@ -873,6 +873,13 @@
       <c r="A76" t="inlineStr">
         <is>
           <t>2026-10-30：DD-94 补十九（空快照基线取可信快照）、二十（构建 REPEATABLE READ、时间轴只算一次、M-10 写入协议）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>2026-10-30：新增 DD-96（fact_call 聚合规则与 call_result 四值）、DD-97（注册表与 mart 的对应、版本后缀）。</t>
         </is>
       </c>
     </row>
@@ -2126,7 +2133,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H96"/>
+  <dimension ref="A1:H98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -6171,6 +6178,90 @@
         </is>
       </c>
     </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>DD-96</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>fact_call 从腿级聚合的规则：首腿未到不建行、末腿未到标 is_complete=false 且发布指标只算完整通话、时间与归属取法、call_result 四值按「先看谁挂的再看有无坐席腿」判定；M-C06/07/11/15 四处口径修正</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>DD-66 定了通话级由腿级聚合、不独立接入，但 fact_call 每列怎么从腿算、呼叫结果怎么派生、首末腿缺失怎么办都没有规则；metrics.yaml 中 M-C07 定义与来源表矛盾、M-C11 用坐席腿的原因码而文档说只在末腿有意义（开发机 2026-10-26 列出的缺口）。</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>见 LD-03 2.4 的十条。要点：call_result 优先级 answered → abandoned（末腿主叫释放，不论在队列还是坐席振铃）→ unanswered_system → ivr_only，未完整为空；transferred / malicious 从结果码移为标志；M-C07 按坐席腿、M-C11 按通话取末腿改占比、M-C06 分母含放弃、M-C15 库内按号码分组只出计数。</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>一、坐席振铃中主叫挂断记 missed。二、未完整通话按现有腿判结果。三、M-C07 按通话平均。四、M-C11 按坐席腿。</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>一、放弃是主叫的行为，与电话当时在哪无关；坐席侧的未接由腿级 M-C12 计，混在结果码里会让一通电话同时「被放弃」又「被漏接」。二、进行中的通话会被判成放弃，第二天又变成应答，日内数字不稳。三、与定义「各腿分别计入」矛盾，且经多个坐席的通话会被低估。四、非末腿的原因码无意义（Q23），按腿统计是噪声。</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>中（结果码是报表分类的基础，dim_call_result 取值一旦有数据即难改；其余为模型规则）</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>DD-66 · DD-91 · DD-95 · LD-02 第 3 章 · LD-03 2.4 · M-C01–M-C15 · if03a</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>DD-97</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>指标注册表不生成 SQL：mart 模型手写，metrics.yaml 以 mart_table / mart_column 指向实现，部署时校验一致；口径版本升级以带后缀的新列实现，旧列保留</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>LD-03 第 5 章定了注册表是口径的权威、库内只读副本，但没定 mart 怎么由它产生、口径版本升级后历史怎么保留；第 8 步要开话务 mart。</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>一、不做 YAML 到 SQL 的生成器：mart 模型由人写 dbt，每条已发布指标在 metrics.yaml 中以 mart_table / mart_column 指向实现列，部署同步 meta.metric_registry 时校验列存在，否则失败。二、metric_version 升级：mart 新增带后缀的列（_v2），旧列保留，注册表按（编码, 版本）指向；历史报表不重算。三、参数型指标的参数记在注册表（M-C05 X 秒默认 20）。四、话务 mart 第一组四张表见 LD-03 第 5 章补充。</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>一、由 metrics.yaml 生成 mart SQL。二、口径升级就地改列、历史重算。</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>一、生成器要覆盖窗口、分母、过滤等全部语义，等于再造一个查询语言，八年维护成本大于收益；校验一致性已足以防止注册表与实现分叉。二、违反 LD-03 第 6 章与 DD-08「去年打印的报表今年重跑一致」。</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>低（约定与校验步骤；不改既有结构）</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>DD-05 · DD-08 · DD-49 · DD-81 · LD-03 第 5、6 章 · LD-04 第 7 章</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H28"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>